<commit_message>
IpsSysAdmin adaptartion to new Wid completed
</commit_message>
<xml_diff>
--- a/DdexInvoicing/WorkingDocs/WidInSmart.xlsx
+++ b/DdexInvoicing/WorkingDocs/WidInSmart.xlsx
@@ -13,8 +13,44 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Автор</author>
+  </authors>
+  <commentList>
+    <comment ref="A22" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="204"/>
+          </rPr>
+          <t>Автор:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="204"/>
+          </rPr>
+          <t xml:space="preserve">
+Главная процедура, вызывается из Смарта только она</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="38">
   <si>
     <t>vWIDTransferIPI</t>
   </si>
@@ -125,13 +161,16 @@
   </si>
   <si>
     <t>Just for pTsk10_Transfer</t>
+  </si>
+  <si>
+    <t>RegisterController.cs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -158,8 +197,23 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -169,6 +223,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -185,11 +245,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -493,7 +554,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -617,6 +678,9 @@
       <c r="A9" t="s">
         <v>8</v>
       </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
       <c r="C9" t="s">
         <v>32</v>
       </c>
@@ -658,6 +722,9 @@
       <c r="A10" t="s">
         <v>10</v>
       </c>
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
       <c r="C10" t="s">
         <v>32</v>
       </c>
@@ -699,6 +766,9 @@
       <c r="A11" t="s">
         <v>11</v>
       </c>
+      <c r="B11" t="s">
+        <v>32</v>
+      </c>
       <c r="C11" t="s">
         <v>32</v>
       </c>
@@ -740,6 +810,9 @@
       <c r="A12" t="s">
         <v>12</v>
       </c>
+      <c r="B12" t="s">
+        <v>32</v>
+      </c>
       <c r="C12" t="s">
         <v>32</v>
       </c>
@@ -778,6 +851,9 @@
       <c r="A13" t="s">
         <v>13</v>
       </c>
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
       <c r="C13" t="s">
         <v>32</v>
       </c>
@@ -813,6 +889,9 @@
       <c r="A14" t="s">
         <v>14</v>
       </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
       <c r="C14" t="s">
         <v>32</v>
       </c>
@@ -848,6 +927,9 @@
       <c r="A15" t="s">
         <v>15</v>
       </c>
+      <c r="B15" t="s">
+        <v>32</v>
+      </c>
       <c r="C15" t="s">
         <v>32</v>
       </c>
@@ -883,6 +965,9 @@
       <c r="A16" t="s">
         <v>7</v>
       </c>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
       <c r="C16" t="s">
         <v>32</v>
       </c>
@@ -918,6 +1003,9 @@
       <c r="A17" t="s">
         <v>16</v>
       </c>
+      <c r="B17" t="s">
+        <v>32</v>
+      </c>
       <c r="C17" t="s">
         <v>32</v>
       </c>
@@ -953,6 +1041,9 @@
       <c r="A18" t="s">
         <v>17</v>
       </c>
+      <c r="B18" t="s">
+        <v>32</v>
+      </c>
       <c r="C18" t="s">
         <v>32</v>
       </c>
@@ -988,6 +1079,9 @@
       <c r="A19" t="s">
         <v>18</v>
       </c>
+      <c r="B19" t="s">
+        <v>32</v>
+      </c>
       <c r="C19" t="s">
         <v>32</v>
       </c>
@@ -1023,6 +1117,9 @@
       <c r="A20" t="s">
         <v>19</v>
       </c>
+      <c r="B20" t="s">
+        <v>32</v>
+      </c>
       <c r="C20" t="s">
         <v>32</v>
       </c>
@@ -1058,6 +1155,9 @@
       <c r="A21" t="s">
         <v>20</v>
       </c>
+      <c r="B21" t="s">
+        <v>32</v>
+      </c>
       <c r="C21" t="s">
         <v>32</v>
       </c>
@@ -1090,8 +1190,11 @@
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="A22" s="4" t="s">
         <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>37</v>
       </c>
       <c r="C22" t="s">
         <v>32</v>
@@ -1128,6 +1231,9 @@
       <c r="A23" t="s">
         <v>22</v>
       </c>
+      <c r="B23" t="s">
+        <v>32</v>
+      </c>
       <c r="C23" t="s">
         <v>32</v>
       </c>
@@ -1163,6 +1269,9 @@
       <c r="A24" t="s">
         <v>23</v>
       </c>
+      <c r="B24" t="s">
+        <v>32</v>
+      </c>
       <c r="C24" t="s">
         <v>32</v>
       </c>
@@ -1198,6 +1307,9 @@
       <c r="A25" t="s">
         <v>24</v>
       </c>
+      <c r="B25" t="s">
+        <v>32</v>
+      </c>
       <c r="C25" t="s">
         <v>32</v>
       </c>
@@ -1233,6 +1345,9 @@
       <c r="A26" t="s">
         <v>25</v>
       </c>
+      <c r="B26" t="s">
+        <v>32</v>
+      </c>
       <c r="C26" t="s">
         <v>32</v>
       </c>
@@ -1268,6 +1383,9 @@
       <c r="A27" t="s">
         <v>26</v>
       </c>
+      <c r="B27" t="s">
+        <v>32</v>
+      </c>
       <c r="C27" t="s">
         <v>32</v>
       </c>
@@ -1303,6 +1421,9 @@
       <c r="A28" t="s">
         <v>6</v>
       </c>
+      <c r="B28" t="s">
+        <v>32</v>
+      </c>
       <c r="C28" t="s">
         <v>32</v>
       </c>
@@ -1338,6 +1459,9 @@
       <c r="A29" t="s">
         <v>27</v>
       </c>
+      <c r="B29" t="s">
+        <v>32</v>
+      </c>
       <c r="C29" t="s">
         <v>32</v>
       </c>
@@ -1378,6 +1502,12 @@
       <c r="A31" t="s">
         <v>6</v>
       </c>
+      <c r="B31" t="s">
+        <v>32</v>
+      </c>
+      <c r="C31" t="s">
+        <v>32</v>
+      </c>
       <c r="D31" t="s">
         <v>7</v>
       </c>
@@ -1430,6 +1560,9 @@
       <c r="A36" t="s">
         <v>27</v>
       </c>
+      <c r="B36" t="s">
+        <v>32</v>
+      </c>
       <c r="C36" t="s">
         <v>32</v>
       </c>
@@ -1464,5 +1597,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>